<commit_message>
Sync See More rebranding source workbook without misplaced Approach section.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/portfolio/see-more-rebranding/See More Rebranding.xlsx
+++ b/public/portfolio/see-more-rebranding/See More Rebranding.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="186">
   <si>
     <t>Chris Bartosik — szablon jednego projektu</t>
   </si>
@@ -26,43 +26,52 @@
     <t>Wrzucasz do folderu projektu</t>
   </si>
   <si>
+    <t>Jak używać</t>
+  </si>
+  <si>
+    <t>Pole</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>Uwagi</t>
+  </si>
+  <si>
     <t>Co robi</t>
   </si>
   <si>
-    <t>Pole</t>
-  </si>
-  <si>
-    <t>Jak używać</t>
-  </si>
-  <si>
-    <t>EN</t>
-  </si>
-  <si>
-    <t>PL</t>
-  </si>
-  <si>
-    <t>ES</t>
-  </si>
-  <si>
-    <t>Uwagi</t>
-  </si>
-  <si>
     <t>1. Skopiuj plik i nazwij np. Epic Realty.xlsx (jeden Excel = jeden projekt).</t>
   </si>
   <si>
+    <t>2. W karcie „Projekt” uzupełnij EN, PL i ES — tylko teksty.</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>3. Wrzuć grafiki do public/portfolio/{folderName}/ (cover, bg, 1.webp, 2.webp…).</t>
+  </si>
+  <si>
     <t>cover.webp / cover.webm / cover.mp4</t>
   </si>
   <si>
     <t>Okładka na liście projektów</t>
   </si>
   <si>
-    <t>2. W karcie „Projekt” uzupełnij EN, PL i ES — tylko teksty.</t>
-  </si>
-  <si>
-    <t>3. Wrzuć grafiki do public/portfolio/{folderName}/ (cover, bg, 1.webp, 2.webp…).</t>
-  </si>
-  <si>
-    <t>Start</t>
+    <t>slug</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>4. Wyślij mi Excel albo wrzuć go do tego folderu — ja wciągam treści.</t>
   </si>
   <si>
     <t>bg.webp</t>
@@ -71,16 +80,10 @@
     <t>Tło hero na stronie projektu</t>
   </si>
   <si>
-    <t>4. Wyślij mi Excel albo wrzuć go do tego folderu — ja wciągam treści.</t>
-  </si>
-  <si>
-    <t>slug</t>
-  </si>
-  <si>
     <t>Co jest automatyczne (nie wpisujesz w Excelu)</t>
   </si>
   <si>
-    <t/>
+    <t>Nazwa pliku projektu, np. epic-realty (→ epic-realty.md). Tylko EN.</t>
   </si>
   <si>
     <t>1.webp</t>
@@ -92,54 +95,51 @@
     <t>Zdjęcia i wideo: cover.webp/mp4, bg.webp, 1.webp (overview), 2.webp / 2.1+2.2… — strona czyta je z folderu. Nie ma pól afterGroup / ścieżek grafik.</t>
   </si>
   <si>
+    <t>folderName</t>
+  </si>
+  <si>
     <t>2.webp, 3.webp, 4.webp…</t>
   </si>
   <si>
     <t>Pełne kadry w galerii (kolejność = numer)</t>
   </si>
   <si>
-    <t>Nazwa pliku projektu, np. epic-realty (→ epic-realty.md). Tylko EN.</t>
-  </si>
-  <si>
     <t>Układ i kolory sekcji: theme idzie automatycznie (dark → light → muted). Overview zawsze jasny. Sekcja Summary / Podsumowanie / Resultado zawsze na końcu.</t>
   </si>
   <si>
+    <t>Folder grafik: public/portfolio/{folderName}/. Zdjęcia bierze strona sama. Tylko EN.</t>
+  </si>
+  <si>
     <t>2.1.webp + 2.2.webp…</t>
   </si>
   <si>
+    <t>Pary pod pełnym kadrem o tym samym numerze</t>
+  </si>
+  <si>
+    <t>order</t>
+  </si>
+  <si>
+    <t>ten Excel (opcjonalnie)</t>
+  </si>
+  <si>
     <t>CAPS (etykiety, tytuły, info) robi CSS na stronie — w Excelu pisz normalnie. Nawiasów [ ] przy labelach nie dopisuj.</t>
   </si>
   <si>
-    <t>Pary pod pełnym kadrem o tym samym numerze</t>
-  </si>
-  <si>
-    <t>folderName</t>
+    <t>Żebym mógł wciągnąć teksty z folderu</t>
+  </si>
+  <si>
+    <t>Kolejność na liście (1, 2, 3…). Mniejsza = wyżej. Tylko EN.</t>
   </si>
   <si>
     <t>Pola tylko EN (żółte i tak wypełnij w kolumnie EN)</t>
   </si>
   <si>
-    <t>ten Excel (opcjonalnie)</t>
-  </si>
-  <si>
-    <t>Żebym mógł wciągnąć teksty z folderu</t>
+    <t>comingSoon</t>
   </si>
   <si>
     <t>slug, folderName, order, comingSoon, categories, year, liveUrl.</t>
   </si>
   <si>
-    <t>Folder grafik: public/portfolio/{folderName}/. Zdjęcia bierze strona sama. Tylko EN.</t>
-  </si>
-  <si>
-    <t>order</t>
-  </si>
-  <si>
-    <t>Kolejność na liście (1, 2, 3…). Mniejsza = wyżej. Tylko EN.</t>
-  </si>
-  <si>
-    <t>comingSoon</t>
-  </si>
-  <si>
     <t>true = Coming soon (wyszarzone), false = aktywny. Tylko EN.</t>
   </si>
   <si>
@@ -431,37 +431,10 @@
     <t>sections.2.label</t>
   </si>
   <si>
-    <t>Approach</t>
-  </si>
-  <si>
-    <t>Podejście</t>
-  </si>
-  <si>
-    <t>Enfoque</t>
-  </si>
-  <si>
     <t>sections.2.title</t>
   </si>
   <si>
-    <t>Leveraging Social Proof and Personal Advisory</t>
-  </si>
-  <si>
-    <t>Wykorzystanie dowodu słuszności i budowanie relacji z twórcami marki</t>
-  </si>
-  <si>
-    <t>Prueba social y enfoque en la relación personal</t>
-  </si>
-  <si>
     <t>sections.2.text</t>
-  </si>
-  <si>
-    <t>I crafted the site architecture to systematically build trust with prospective buyers. Moving away from cold corporate real estate models, I focused the user journey on a curated advisory philosophy ("Curadores, no solo agentes"). Key pages highlight the founders' profiles, giving clients direct access to senior leadership. To reinforce credibility, I introduced high-end gallery sliders showcasing premier developments and integrated a testimonial module ("La voz de nuestros clientes") across strategic touchpoints.</t>
-  </si>
-  <si>
-    <t>Całą strukturę serwisu zaplanowałem tak, aby krok po kroku budować zaufanie potencjalnego inwestora. Zamiast tworzyć anonimowy portal, w centrum postawiłem podejście kuratorskie (Curadores, no solo agentes) oraz bezpośrednią relację z założycielami agencji. Na podstronie „O nas” oraz w kluczowych sekcjach wyeksponowałem sylwetki właścicieli, co skraca dystans i eliminuje zbędne procesy korporacyjne. Dopełnieniem tej strategii stała się zaprojektowana przeze mnie sekcja z płynnie zmieniającymi się zdjęciami najlepszych inwestycji oraz moduł opinii klientów (La voz de nuestros clientes).</t>
-  </si>
-  <si>
-    <t>Planifiqué la arquitectura del sitio para generar confianza de forma progresiva. En lugar de un portal impersonal, centré la narrativa en un enfoque de asesoría boutique ("Curadores, no solo agentes") y en la cercanía con los fundadores. En las secciones principales y la página "Nosotros" destaqué las figuras de los líderes de la firma, habilitando un trato directo. Como refuerzo de credibilidad, integré galerías dinámicas de proyectos destacados y un módulo de testimonios ("La voz de nuestros clientes") en puntos clave del recorrido.</t>
   </si>
   <si>
     <t>Sekcja 04</t>
@@ -1068,7 +1041,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1128,7 +1101,7 @@
     </row>
     <row r="5" ht="39.75" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1158,7 +1131,7 @@
     </row>
     <row r="6" ht="39.75" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1218,7 +1191,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1248,7 +1221,7 @@
     </row>
     <row r="10" ht="39.75" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1278,7 +1251,7 @@
     </row>
     <row r="11" ht="39.75" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1308,7 +1281,7 @@
     </row>
     <row r="12" ht="39.75" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1338,7 +1311,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1368,7 +1341,7 @@
     </row>
     <row r="15" ht="39.75" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -2406,16 +2379,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -2440,22 +2413,22 @@
     </row>
     <row r="2" ht="31.5" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -2480,22 +2453,22 @@
     </row>
     <row r="3" ht="31.5" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -2520,22 +2493,22 @@
     </row>
     <row r="4" ht="31.5" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -2560,19 +2533,19 @@
     </row>
     <row r="5" ht="31.5" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="12" t="b">
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>41</v>
@@ -2600,7 +2573,7 @@
     </row>
     <row r="6" ht="31.5" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>42</v>
@@ -2609,10 +2582,10 @@
         <v>43</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>44</v>
@@ -3081,10 +3054,10 @@
         <v>90</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>91</v>
@@ -3477,15 +3450,9 @@
       <c r="B28" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="E28" s="17" t="s">
-        <v>140</v>
-      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="17"/>
       <c r="F28" s="5" t="s">
         <v>112</v>
       </c>
@@ -3515,17 +3482,11 @@
         <v>136</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>144</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="C29" s="12"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="15"/>
       <c r="F29" s="5" t="s">
         <v>117</v>
       </c>
@@ -3555,17 +3516,11 @@
         <v>136</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>148</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="17"/>
       <c r="F30" s="5" t="s">
         <v>122</v>
       </c>
@@ -3592,19 +3547,19 @@
     </row>
     <row r="31" ht="31.5" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>112</v>
@@ -3632,19 +3587,19 @@
     </row>
     <row r="32" ht="24.0" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>117</v>
@@ -3672,19 +3627,19 @@
     </row>
     <row r="33" ht="31.5" customHeight="1">
       <c r="A33" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>158</v>
-      </c>
       <c r="C33" s="12" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>122</v>
@@ -3712,19 +3667,19 @@
     </row>
     <row r="34" ht="31.5" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>112</v>
@@ -3752,19 +3707,19 @@
     </row>
     <row r="35" ht="24.0" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>117</v>
@@ -3792,19 +3747,19 @@
     </row>
     <row r="36" ht="31.5" customHeight="1">
       <c r="A36" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>171</v>
-      </c>
       <c r="D36" s="16" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>122</v>
@@ -3832,19 +3787,19 @@
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D37" s="24" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>112</v>
@@ -3872,19 +3827,19 @@
     </row>
     <row r="38" ht="24.0" customHeight="1">
       <c r="A38" s="5" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>117</v>
@@ -3912,19 +3867,19 @@
     </row>
     <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D39" s="24" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>122</v>
@@ -3952,19 +3907,19 @@
     </row>
     <row r="40" ht="31.5" customHeight="1">
       <c r="A40" s="5" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F40" s="5" t="s">
         <v>112</v>
@@ -3992,19 +3947,19 @@
     </row>
     <row r="41" ht="24.0" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D41" s="24" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E41" s="25" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>117</v>
@@ -4032,19 +3987,19 @@
     </row>
     <row r="42" ht="31.5" customHeight="1">
       <c r="A42" s="5" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>122</v>
@@ -4072,19 +4027,19 @@
     </row>
     <row r="43" ht="31.5" customHeight="1">
       <c r="A43" s="5" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>112</v>
@@ -4112,19 +4067,19 @@
     </row>
     <row r="44" ht="24.0" customHeight="1">
       <c r="A44" s="5" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>117</v>
@@ -4152,19 +4107,19 @@
     </row>
     <row r="45" ht="31.5" customHeight="1">
       <c r="A45" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B45" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>191</v>
-      </c>
       <c r="C45" s="12" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>122</v>
@@ -5174,7 +5129,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -5203,10 +5158,10 @@
     </row>
     <row r="2" ht="27.75" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -5235,10 +5190,10 @@
     </row>
     <row r="3" ht="27.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -5267,10 +5222,10 @@
     </row>
     <row r="4" ht="27.75" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -5299,10 +5254,10 @@
     </row>
     <row r="5" ht="27.75" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -5331,10 +5286,10 @@
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
@@ -5366,7 +5321,7 @@
         <v>34</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>

</xml_diff>